<commit_message>
Stabilize Printify cover gate and LAN resume state
</commit_message>
<xml_diff>
--- a/Database/Etsy_listing.xlsx
+++ b/Database/Etsy_listing.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:E241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,7 +583,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:13 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2419,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:53 PM</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3175,7 +3175,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:14 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3715,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4327,7 +4327,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4399,7 +4399,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4435,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4615,7 +4615,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4903,7 +4903,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4939,7 +4939,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5047,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5083,7 +5083,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5155,7 +5155,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5443,7 +5443,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5587,7 +5587,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5623,7 +5623,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:54 PM</t>
         </is>
       </c>
     </row>
@@ -5659,7 +5659,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:15 PM</t>
+          <t>4/29/2026  1:28:55 PM</t>
         </is>
       </c>
     </row>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:16 PM</t>
+          <t>4/29/2026  1:28:55 PM</t>
         </is>
       </c>
     </row>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:16 PM</t>
+          <t>4/29/2026  1:28:55 PM</t>
         </is>
       </c>
     </row>
@@ -5767,7 +5767,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:16 PM</t>
+          <t>4/29/2026  1:28:55 PM</t>
         </is>
       </c>
     </row>
@@ -5803,7 +5803,3283 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>4/28/2026  10:49:16 PM</t>
+          <t>4/29/2026  1:28:55 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0001</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0001
+Timestamp: 2026-04-27 00:22:26.281000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Astral Archive Gateway of Temporal Wisdom
+MJ_Prompt: A towering celestial gate forged from luminous moonstone and imperial jade rising before a suspended chronicle library, ancient leather-bound manuscripts spiraling through the dimensional portal, ethereal ink-wash cosmos clouds blending with aged parchment particles, levitating talisman shards etched with brass astronomical symbols, cinematic chiaroscuro lighting with jade radiance, dark academia aesthetic, ultra-detailed moonstone crystalline texture and brass clockwork mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: celestial gateway, moonstone architecture, imperial jade portal, floating library, dark academia, ancient manuscripts, brass clockwork, mystical knowledge, temporal wisdom, ethereal lighting, collectible artifact, mentor-grade design, bioluminescent glow
+Status: Defeated_Timeout
+</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:23:28 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0002</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0002
+Timestamp: 2026-04-27 00:22:31.519000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Obsidian Threshold of Eternal Scholarship
+MJ_Prompt: A monumental threshold constructed from polished moonstone and deep imperial jade positioned before a hovering repository of wisdom, weathered calfskin tomes swirling through the mystical passage, cosmic ink-wash mists interweaving with manuscript essence, suspended brass-inscribed charm fragments, cinematic chiaroscuro lighting with jade luminescence, dark academia aesthetic, ultra-detailed moonstone surface patterns and brass mechanical elements, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: obsidian threshold, eternal scholarship, jade architecture, floating tomes, dark academia decor, mystical passage, brass inscriptions, moonstone polish, cosmic atmosphere, premium artifact, mentor wisdom, museum lighting
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0002_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:23:36 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0003</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0003
+Timestamp: 2026-04-27 00:22:35.869000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Serpentine Portal of Alchemical Texts
+MJ_Prompt: A serpentine gateway crafted from iridescent moonstone and imperial jade standing before a levitating archive chamber, ancient leather volumes cascading through the portal vortex, nebulous ink-wash clouds merging with aged paper dust, floating brass talisman pieces with engraved hermetic symbols, cinematic chiaroscuro lighting with jade phosphorescence, dark academia aesthetic, ultra-detailed moonstone iridescence and brass gear mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: serpentine portal, alchemical texts, iridescent moonstone, jade gateway, hermetic symbols, levitating archive, brass mechanisms, dark academia art, nebulous atmosphere, collectible design, mentor-grade quality, phosphorescent jade
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0003_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:23:45 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Acrylic-Academia-0001</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Academia-0001
+Timestamp: 2026-04-29 16:02:30.291000
+Category: Academia
+Product_Type: Acrylic
+Style: Academia Mentor-Grade
+Title: Astrolabe Compass Ritual Disc
+MJ_Prompt: A mechanical astrolabe ritual disc with Moonstone rotating rings and Imperial Jade directional markers, floating compass rose center with glowing constellation pathways, suspended brass gears and crystalline fragments, ink-wash nebula atmosphere swirling through openwork design, isolated on white background, ethereal backlighting, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, brass mechanisms, ink-wash nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: astrolabe compass, celestial navigation, Moonstone ritual disc, Imperial Jade markers, astronomical instrument, academia collectible, mentor-grade artifact, brass mechanism, constellation pathways, premium acrylic art, gallery object, translucent depth, bioluminescent glow, handcrafted precision, museum-grade design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Academia-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:09:39 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0081</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0081
+Timestamp: 2026-04-29 16:02:04.034000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Plague Doctor Raven Skull
+MJ_Prompt: An ornate plague doctor raven skull with elongated brass beak apparatus, Corroded Iron rivets and hinges, Kintsugi gold veins sealing bone fractures, toxic amber bioluminescent vapor seeping from eye sockets, grimdark industrial aesthetic, dramatic underlighting, sharp focus, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: aged bone, Corroded Iron, brass oxidized metal, Kintsugi gold, toxic amber bioluminescence, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: plague doctor skull, grimdark alchemy, bioluminescent artifact, kintsugi gold repair, corroded brass apparatus, toxic amber glow, raven bone relic, industrial gothic decor, premium acrylic art, collectible dark fantasy, mentor-grade design, ray traced depth, museum quality sculpture
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0081_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:14:58 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0001</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0001
+Timestamp: 2026-04-29 16:02:59.376000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Crane Guardian Mechanism
+MJ_Prompt: A mechanical origami crane with folding wings of brushed moonstone and imperial jade, clockwork joints with aquamarine crystal hinges, ink-wash nebula patterns flowing across wing panels, floating talisman fragments orbiting the body, zen-cyber aesthetic, soft blue and violet bioluminescence, celestial mist, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Aquamarine, Brushed Metal, Clockwork Brass, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: mechanical crane, origami sculpture, moonstone wings, jade clockwork, aquamarine crystals, zen cyberpunk, bioluminescent art, floating fragments, celestial mist, premium acrylic block, collectible artifact, translucent depth, museum grade lighting
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:15:27 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0081</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0081
+Timestamp: 2026-04-29 15:58:38.218000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Celestial Armillary Navigation Sphere
+MJ_Prompt: An ornate armillary sphere with rotating brass rings orbiting a central Starlight Jade core, concentric Obsidian bands etched with constellation maps, floating crystalline navigation markers suspended in mid-rotation, dark academia aesthetic with astronomical precision, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, sharp focus, wide cinematic angle, dramatic side lighting, hyper-detailed mentor-grade object design, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: celestial navigation sphere, armillary sphere art, astronomical instrument poster, dark academia decor, constellation map wall art, brass and jade celestial globe, vintage astronomy print, scholar study decoration, astrological navigation tool, mentor-grade collectible, premium vertical poster, museum-quality celestial art
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0081_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:30:39 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0082</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0082
+Timestamp: 2026-04-29 15:59:51.741000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Celestial Armillary Codex
+MJ_Prompt: An ornate armillary sphere with rotating brass rings surrounding an open ancient book with constellation maps, pages made of translucent Amber sheets with glowing star charts, floating golden stardust particles orbiting the rings, warm academic library lighting, mechanical gears visible at joints, crystalline navigation tools embedded in rings, aged brass patina with micro-engraved astronomical symbols, layered translucent depth, subtle internal bioluminescent glow from book pages, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: astrological globe poster, celestial navigation art, brass armillary sphere, academic astronomy decor, amber constellation map, vintage scientific instrument, museum quality wall art, astrology scholar gift, mechanical cosmos print, golden stardust design, antique astronomy poster
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0082_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:30:55 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0083</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0083
+Timestamp: 2026-04-29 15:59:56.687000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Cosmic Lotus Observatory
+MJ_Prompt: A blooming mechanical lotus flower with brass petals that unfold to reveal crystalline star charts, center core made of translucent Amber with glowing celestial coordinates, golden stardust emanating from stamens, each petal engraved with zodiac symbols and planetary orbits, warm academic lighting, sharp focus, botanical-astronomical hybrid design, aged brass with kintsugi-like amber veins, floating accent fragments, layered translucent depth, subtle internal bioluminescent glow, refined handcrafted edge bevels, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: botanical astronomy art, mechanical lotus poster, brass flower celestial, academic astrology decor, amber star chart, steampunk botanical print, cosmic lotus wall art, zodiac flower design, golden stardust botanical, museum grade nature astronomy
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0083_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:31:18 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0084</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0084
+Timestamp: 2026-04-29 16:00:01.204000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Astrolabe Chalice Relic
+MJ_Prompt: An ancient ceremonial chalice with astrolabe mechanisms integrated into the cup, vessel body made of translucent Amber with suspended glowing star maps, brass rim engraved with celestial coordinates, golden stardust swirling inside the cup, ornate brass base with rotating zodiac rings, crystalline charts embedded in stem, warm academic lighting, sharp focus, ritual instrument design, aged brass patina with micro-engraved constellations, layered translucent depth, subtle internal bioluminescent glow, visible handcrafted edge bevels, floating accent fragments, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: astrolabe chalice art, ceremonial astronomy vessel, brass ritual cup, academic astrology artifact, amber star chart goblet, celestial instrument poster, museum quality chalice, golden stardust vessel, antique astronomy relic, zodiac chalice print
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0084_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:31:33 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0082</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0082
+Timestamp: 2026-04-29 16:02:08.302000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Withered Mandrake Root Chamber
+MJ_Prompt: A preserved withered mandrake root suspended in geometric glass terrarium chamber, Corroded Iron frame structure, Kintsugi gold veins running through cracked root system, toxic amber bioluminescent preservative fluid pooling at base, grimdark industrial aesthetic, dramatic underlighting, sharp focus, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: desiccated botanical specimen, Corroded Iron, laboratory glass, Kintsugi gold, toxic amber bioluminescence, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: alchemical terrarium, preserved mandrake root, grimdark botanical specimen, corroded iron frame, kintsugi gold veins, toxic amber fluid, laboratory relic, industrial apothecary art, premium vertical acrylic, gallery collectible, bioluminescent preservation, mentor-grade design, ray traced glass
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0082_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:15:05 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0002</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0002
+Timestamp: 2026-04-29 16:03:03.634000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Ritual Bell Shrine
+MJ_Prompt: An ancient meditation bell with body crafted from brushed moonstone and imperial jade panels, clockwork brass suspension mount, glowing aquamarine prayer beads spiraling around the bell, ink-wash nebula patterns etched into surface, floating talisman fragments circling the artifact, zen-cyber aesthetic, soft blue and violet bioluminescence, celestial mist, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Aquamarine, Brushed Metal, Clockwork Brass, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: meditation bell, ritual instrument, moonstone panels, jade craftsmanship, prayer beads, aquamarine glow, zen architecture, floating talismans, celestial artifact, premium collectible, translucent layers, museum quality, handcrafted details
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0002_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:15:35 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0003</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0003
+Timestamp: 2026-04-29 16:03:07.975000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Pagoda Fragment Relic
+MJ_Prompt: A floating miniature pagoda tower section with walls of brushed moonstone and imperial jade, clockwork brass structural framework, aquamarine crystal windows glowing from within, ink-wash nebula patterns swirling through interior chambers, floating talisman fragments orbiting the structure, zen-cyber aesthetic, soft blue and violet bioluminescence, celestial mist, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Aquamarine, Brushed Metal, Clockwork Brass, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: pagoda architecture, floating tower, moonstone walls, jade framework, aquamarine windows, clockwork brass, zen relic, celestial structure, bioluminescent interior, premium art object, layered depth, gallery collectible, architectural fragment
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0003_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:15:43 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0085</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0085
+Timestamp: 2026-04-29 16:00:05.866000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Orrery Lighthouse Beacon
+MJ_Prompt: A miniature lighthouse tower with mechanical orrery planets orbiting around its beacon chamber, central light made of translucent Amber with glowing star charts projecting outward, brass planetary rings rotating at different levels, golden stardust trails marking orbital paths, crystalline navigation lenses, warm academic lighting, architectural relic design, aged brass with micro-engraved latitude lines, layered translucent depth showing internal gear mechanisms, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: orrery lighthouse poster, architectural astronomy art, brass planetary beacon, celestial navigation tower, amber star chart light, mechanical solar system, academic astrology architecture, golden stardust orbital, museum lighthouse print, vintage orrery design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0085_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:31:53 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0091</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0091
+Timestamp: 2026-04-29 16:01:36.024000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Jade Lotus Celestial Mechanism
+MJ_Prompt: A delicate mechanical lotus flower with petals carved from imperial jade and moonstone glass, rotating brass gear core with copper wire stamens, ink-wash constellation patterns etched on translucent petals, floating talisman paper fragments orbiting the bloom, hand-blown glass dewdrops suspended on wire tendrils, illuminated by soft candlelight, academia aesthetic, primary material system: Hand-blown Glass, Moonstone Glass, Imperial Jade, Copper Wire, Talisman Paper, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: jade lotus mechanism, glass orrery art, celestial botanical sculpture, hand-blown glass flower, copper wire botanical, academia glass art, moonstone petal design, mechanical flower poster, oriental glass craft, museum-grade botanical art, translucent jade sculpture, cinematic wall art, premium vertical poster
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0091_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:32:09 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Acrylic-Academia-0003</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Academia-0003
+Timestamp: 2026-04-29 16:02:40.260000
+Category: Academia
+Product_Type: Acrylic
+Style: Academia Mentor-Grade
+Title: Celestial Orrery Tree Bonsai
+MJ_Prompt: A miniature celestial bonsai tree with Moonstone trunk and branches forming orbital paths, Imperial Jade leaves shaped as planetary bodies with glowing astronomical symbols, roots suspended in crystalline soil with floating talisman fragments and stardust particles, ink-wash nebula atmosphere pooling around base, isolated on white background, ethereal backlighting, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, crystalline minerals, ink-wash nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: orrery bonsai, celestial tree, Moonstone trunk, Imperial Jade planets, botanical astronomy, miniature cosmos, academia plant, orbital branches, crystalline roots, premium acrylic sculpture, mentor-grade horticulture, translucent foliage, bioluminescent leaves, gallery botanical art
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Academia-0003_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:09:49 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0083</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0083
+Timestamp: 2026-04-29 16:02:12.509000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Ritual Censer Thurible
+MJ_Prompt: An ancient ritual censer thurible with perforated Corroded Iron shell, cracked heavy glass viewing window, Kintsugi gold veins sealing fractures, toxic amber bioluminescent incense smoke billowing from ornate vents, heavy chain suspension system, grimdark industrial aesthetic, dramatic underlighting, sharp focus, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, cracked glass, Kintsugi gold, toxic amber bioluminescence, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: grimdark thurible, ritual censer artifact, corroded iron incense burner, kintsugi gold repair, toxic amber smoke, bioluminescent vessel, ceremonial relic, industrial gothic design, premium acrylic block, mentor-grade collectible, ray traced depth, museum quality art
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0083_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:15:12 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0004</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0004
+Timestamp: 2026-04-29 16:03:12.047000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Koi Automaton Spirit
+MJ_Prompt: A mechanical koi fish with segmented armor plates of brushed moonstone and imperial jade, clockwork brass joints and gears visible at articulation points, aquamarine crystal scales catching light, ink-wash nebula patterns flowing along body, floating talisman fragments following the fish, zen-cyber aesthetic, soft blue and violet bioluminescence, celestial mist, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Aquamarine, Brushed Metal, Clockwork Brass, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: mechanical koi, automaton fish, moonstone armor, jade segments, aquamarine scales, clockwork creature, zen cyberpunk, bioluminescent design, floating talismans, premium sculpture, translucent materials, collectible art, handcrafted details
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0004_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:15:51 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0005</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0005
+Timestamp: 2026-04-29 16:03:16.163000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Incense Vessel Constellation
+MJ_Prompt: An ornate incense burner with spherical body of brushed moonstone and imperial jade segments, clockwork brass lid mechanism with rotating celestial patterns, aquamarine crystal smoke vents glowing softly, ink-wash nebula patterns emerging as ethereal vapor, floating talisman fragments suspended above the vessel, zen-cyber aesthetic, soft blue and violet bioluminescence, celestial mist, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Aquamarine, Brushed Metal, Clockwork Brass, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: incense burner, ritual vessel, moonstone sphere, jade segments, aquamarine vents, clockwork mechanism, zen container, celestial vapor, bioluminescent glow, premium artifact, translucent design, museum collectible, handcrafted luxury
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0005_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:15:59 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Poster-Zen-0001</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Zen-0001
+Timestamp: 2026-04-29 16:00:55.281000
+Category: Zen
+Product_Type: Poster
+Style: Zen Mentor-Grade
+Title: Celestial Gate of Jade Mist
+MJ_Prompt: A miniature floating mountain with a bonsai tree made of Imperial Green Jade framed by a Moonstone torii gate, crystalline waterfalls falling into clouds, obsidian rock base, ink-wash nebula backdrop, floating talisman fragments, ethereal zen aesthetic, soft morning mist lighting, isolated on white background, ultra-wide angle, hyper-detailed mentor-grade object design, primary material system: Imperial Green Jade, Moonstone, Floating Obsidian, Talisman Fragments, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: zen bonsai wall art, jade floating mountain poster, moonstone torii gate, celestial asian decor, premium vertical poster, ethereal jade tree, floating mountain art, zen meditation decor, oriental mystical poster, translucent jade artwork
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Zen-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:32:34 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Poster-Zen-0002</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Zen-0002
+Timestamp: 2026-04-29 16:01:00.572000
+Category: Zen
+Product_Type: Poster
+Style: Zen Mentor-Grade
+Title: Phoenix Flame Ritual Vessel
+MJ_Prompt: An ornate ceremonial incense burner shaped as a rising phoenix crafted from Imperial Green Jade wings with Moonstone flame accents, floating obsidian smoke wisps, talisman fragments orbiting the vessel, carved feather detail with micro-engraved surface relief, ethereal zen aesthetic, soft morning mist lighting, isolated on white background, ultra-wide angle, hyper-detailed mentor-grade object design, primary material system: Imperial Green Jade, Moonstone, Floating Obsidian, Talisman Fragments, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: phoenix incense burner art, jade ritual vessel poster, ceremonial zen decor, moonstone flame phoenix, oriental vessel artwork, floating obsidian smoke, premium jade phoenix, ritual object wall art, asian ceremonial decor, translucent phoenix poster
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Zen-0002_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:33:11 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Poster-Zen-0003</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Zen-0003
+Timestamp: 2026-04-29 16:01:04.761000
+Category: Zen
+Product_Type: Poster
+Style: Zen Mentor-Grade
+Title: Lotus Mandala Seal Stone
+MJ_Prompt: An ancient circular talisman seal carved with blooming lotus mandala pattern in Imperial Green Jade, Moonstone prayer beads wrapped around edges, floating obsidian meditation stones, ink-wash nebula backdrop, sacred geometry micro-engravings, ethereal zen aesthetic, soft morning mist lighting, isolated on white background, ultra-wide angle, hyper-detailed mentor-grade object design, primary material system: Imperial Green Jade, Moonstone, Floating Obsidian, Talisman Fragments, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: lotus mandala seal art, jade talisman poster, sacred geometry decor, moonstone prayer beads, zen meditation seal, oriental mandala artwork, floating stone talisman, premium jade seal, buddhist symbol poster, translucent lotus art
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Zen-0003_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:33:26 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0006</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0006
+Timestamp: 2026-04-29 16:03:28.318000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Jade Phoenix Incense Altar
+MJ_Prompt: A ceremonial phoenix sculpture carved from imperial jade perched on a floating incense altar, wings spread in flight pose with moonstone feather inlays, rising smoke forming zen calligraphy symbols, ink-wash nebula background, scattered lotus petal fragments, zen aesthetic, soft celestial glow, bamboo silhouette fading into mist, , 3D relief effect, solid white background isolated on white background, hyper-detailed mentor-grade object design, primary material system: Imperial Jade, Moonstone, Raku Pottery Base, Emerald Smoke, Ink-Wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: jade phoenix sculpture, zen incense altar, moonstone inlay art, imperial jade carving, ceremonial tea decor, ink-wash nebula aesthetic, floating lotus fragments, bioluminescent glow, kintsugi vein detail, museum-grade collectible, mentor-grade zen object, celestial phoenix totem, raku pottery base, translucent depth acrylic
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0006_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:16:08 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0007</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0007
+Timestamp: 2026-04-29 16:03:34.002000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Sacred Lotus Meditation Bell
+MJ_Prompt: An ancient bronze meditation bell shaped as blooming lotus flower with rough raku pottery clapper, moonstone dewdrops on petals, imperial jade stem wrapped in silk cord, sound wave ripples visualized as ink-wash nebula rings, floating prayer beads orbiting, zen aesthetic, soft celestial glow, bamboo forest silhouette fading into mist, , 3D relief effect, solid white background isolated on white background, hyper-detailed mentor-grade object design, primary material system: Aged Bronze, Rough Raku Pottery, Moonstone, Imperial Jade, Ink-Wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: lotus meditation bell, bronze ritual instrument, raku pottery clapper, moonstone dewdrops, sacred sound visualization, zen prayer beads, imperial jade stem, ink-wash sound waves, bioluminescent lotus art, handcrafted bronze bell, kintsugi detail work, celestial glow artifact, museum-quality bell sculpture, translucent acrylic depth
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0007_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:16:16 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0008</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0008
+Timestamp: 2026-04-29 16:03:39.649000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Celestial Bonsai Moon Garden
+MJ_Prompt: A miniature celestial bonsai tree growing from crescent moon-shaped rough raku pottery vessel, branches made of twisted imperial jade wire with moonstone blossoms, roots visible through translucent vessel walls, ink-wash nebula soil glowing softly, floating stone lantern fragments, zen aesthetic, soft celestial glow, bamboo forest silhouette fading into mist, , 3D relief effect, solid white background isolated on white background, hyper-detailed mentor-grade object design, primary material system: Rough Raku Pottery, Imperial Jade Wire, Moonstone Blossoms, Luminous Nebula Soil, Ink-Wash Mist, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: celestial bonsai sculpture, crescent moon vessel, imperial jade branches, moonstone blossom tree, raku pottery planter, luminous nebula soil, floating lantern fragments, translucent root system, zen garden miniature, bioluminescent botanical art, kintsugi vessel detail, museum-grade bonsai object, handcrafted jade wire, premium acrylic composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0008_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:16:24 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Poster-Zen-0004</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Zen-0004
+Timestamp: 2026-04-29 16:01:22.158000
+Category: Zen
+Product_Type: Poster
+Style: Zen Mentor-Grade
+Title: Celestial Compass Relic
+MJ_Prompt: An ornate celestial compass made of Imperial Green Jade with obsidian directional markers and amethyst constellation inlays, crystalline water droplets suspended in rotating rings, ethereal zen aesthetic, twilight purple-gold lighting, isolated on white background, three-quarter elevated view, hyper-detailed mentor-grade object design, primary material system: Imperial Green Jade, Floating Obsidian, Amethyst, Crystalline Water, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: zen celestial compass, jade navigation relic, amethyst constellation art, obsidian directional markers, ethereal compass design, twilight mystical artifact, premium spiritual decor, bioluminescent jade object, museum-grade zen art, floating crystal compass, handcrafted celestial instrument, purple-gold lighting poster, translucent jade composition, high-end zen collectible
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Zen-0004_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:33:41 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Poster-Zen-0005</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Zen-0005
+Timestamp: 2026-04-29 16:01:26.639000
+Category: Zen
+Product_Type: Poster
+Style: Zen Mentor-Grade
+Title: Phoenix Rebirth Vessel
+MJ_Prompt: An ancient ceremonial vessel shaped as an ascending phoenix with wings made of Imperial Green Jade feathers, obsidian talons gripping amethyst flame base, crystalline water flowing upward in spiral patterns, ethereal zen aesthetic, twilight purple-gold lighting, isolated on white background, dynamic upward spiral composition, hyper-detailed mentor-grade object design, primary material system: Imperial Green Jade, Floating Obsidian, Amethyst, Crystalline Water, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium matte vertical poster composition, full frame, cinematic lighting, edge-to-edge composition, immersive environment, 12x18 wall art format, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: zen phoenix vessel, jade rebirth sculpture, amethyst flame artifact, obsidian talon design, crystalline water spiral, ethereal bird container, twilight ceremonial art, premium spiritual vessel, bioluminescent phoenix object, museum-grade zen collectible, ascending jade wings, purple-gold mystical poster, translucent feather composition, high-end rebirth symbol
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Zen-0005_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:33:54 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Acrylic-Academia-0005</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Academia-0005
+Timestamp: 2026-04-29 16:02:48.865000
+Category: Academia
+Product_Type: Acrylic
+Style: Academia Mentor-Grade
+Title: Alchemical Star Flask Vessel
+MJ_Prompt: An ornate alchemical flask vessel with Moonstone body and Imperial Jade stopper, interior filled with swirling liquid cosmos containing miniature galaxies and floating talisman fragments, geometric sacred patterns etched into surface with glowing star coordinates, suspended droplets of luminous nebula essence, ink-wash nebula atmosphere emanating from opening, isolated on white background, ethereal backlighting, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, liquid cosmos, ink-wash nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: alchemical flask, star vessel, Moonstone container, Imperial Jade stopper, liquid cosmos, celestial potion, academia alchemy, contained universe, sacred geometry, premium acrylic bottle, mentor-grade glasswork, translucent elixir, bioluminescent fluid, gallery apothecary art
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Academia-0005_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:09:55 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0085</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0085
+Timestamp: 2026-04-29 16:02:20.451000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Alchemist's Divination Compass
+MJ_Prompt: An ornate alchemist's divination compass with Corroded Iron housing and cracked glass face, Kintsugi gold veins repairing fracture lines, toxic amber bioluminescent liquid filling internal chambers behind rotating brass needle mechanisms, grimdark industrial aesthetic, dramatic underlighting, sharp focus, macro photography, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, cracked glass, Kintsugi gold, brass mechanisms, toxic amber bioluminescence, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: alchemical compass, divination instrument, grimdark navigation tool, corroded iron housing, kintsugi gold repair, toxic amber liquid, bioluminescent brass mechanism, industrial occult art, premium acrylic display, mentor-grade design, ray traced glass, gallery collectible talisman
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0085_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:15:20 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0009</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0009
+Timestamp: 2026-04-29 16:04:01.828000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Whispering Bamboo Flute
+MJ_Prompt: A floating shakuhachi bamboo flute made of aged bamboo with natural nodes and grain texture in warm honey tones, ethereal mist spiraling from the mouthpiece forming delicate kanji characters, zen garden stones arranged in contemplative pattern below, soft morning light filtering through translucent fog, serene meditation aesthetic, wisps of pale jade vapor, , 3D relief effect, solid white background isolated on white background, hyper-detailed mentor-grade object design, primary material system: Aged Bamboo, Honey Tones, Jade Vapor, Morning Light, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: zen bamboo flute meditation, shakuhachi spiritual art, japanese bamboo instrument, contemplative music decor, mindfulness ritual object, asian meditation gift, bamboo grain texture, ethereal mist design, serene morning light, premium zen collectible, museum-grade oriental art, handcrafted bamboo aesthetic, tranquil spiritual decor
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0009_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:16:32 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Acrylic-Zen-0010</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Zen-0010
+Timestamp: 2026-04-29 16:04:08.119000
+Category: Zen
+Product_Type: Acrylic
+Style: Zen Mentor-Grade
+Title: Lotus Seed Pod Vessel
+MJ_Prompt: A floating dried lotus seed pod vessel in weathered terracotta and dusty sage tones, intricate honeycomb pattern of seed chambers visible, delicate golden pollen particles suspended in air around it, reflected in still water surface below creating mirror symmetry, warm sunset amber glow, botanical zen aesthetic, traces of burnt umber patina, , 3D relief effect, solid white background isolated on white background, hyper-detailed mentor-grade object design, primary material system: Dried Lotus Pod, Terracotta Patina, Golden Pollen, Amber Reflection, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, premium vertical acrylic photo block composition, 3D depth, refractive light, internal glow, ray tracing, gallery collectible art object, --ar 5:7 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: lotus seed pod art, botanical zen decor, dried lotus vessel, nature meditation object, organic texture design, terracotta patina aesthetic, golden pollen particles, sunset reflection art, sacred botanical gift, premium nature collectible, museum-grade botanical art, contemplative seed pod, tranquil organic sculpture
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Zen-0010_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:16:39 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0001</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0001
+Timestamp: 2026-04-27 00:25:06.154000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Crimson Warden's Soul Cage
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron, containing a trapped swirling crimson spirit flame, light refracting through cracked ghostly ruby glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly ruby glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Ruby Glass, Crimson Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: gothic lantern, soul cage, crimson flame, wrought iron, grimdark decor, spirit vessel, collectible artifact, haunted lantern, ruby glass, refractive light, internal glow, premium fantasy
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0001_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:10:03 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0004</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0004
+Timestamp: 2026-04-27 00:25:15.945000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Shadowbound Sentinel's Beacon
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with skeletal framework, containing a trapped swirling ice-blue spirit flame, light refracting through cracked ghostly frost glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly frost glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Frost Glass, Ice-Blue Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: sentinel beacon, ice-blue flame, frost glass, skeletal lantern, grimdark design, spirit light, gothic collectible, shadowbound artifact, refractive glass, internal glow, premium fantasy
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0004_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:10:11 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0005</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0005
+Timestamp: 2026-04-27 00:25:18.787000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Necromancer's Soul Reliquary
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with skull motifs, containing a trapped swirling green spirit flame, light refracting through cracked ghostly emerald glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly emerald glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Emerald Glass, Green Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: necromancer lantern, soul reliquary, green flame, emerald glass, skull motif, grimdark collectible, spirit vessel, gothic artifact, refractive light, bioluminescent core, premium dark fantasy
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0005_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:10:19 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0006</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0006
+Timestamp: 2026-04-27 00:25:22.086000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Voidwalker's Eternal Lamp
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with chain suspension, containing a trapped swirling purple spirit flame, light refracting through cracked ghostly obsidian glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly obsidian glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Obsidian Glass, Purple Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: voidwalker lamp, purple flame, obsidian glass, chain lantern, grimdark decor, eternal light, gothic collectible, spirit container, refractive depth, internal radiance, premium artifact
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0006_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:10:27 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0007</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0007
+Timestamp: 2026-04-27 00:25:25.470000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Banshee's Wailing Lantern
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with thorn patterns, containing a trapped swirling silver spirit flame, light refracting through cracked ghostly moonstone glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly moonstone glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Moonstone Glass, Silver Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: banshee lantern, silver flame, moonstone glass, thorn pattern, grimdark fantasy, wailing light, gothic artifact, spirit beacon, refractive glass, luminescent core, premium collectible
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0007_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:10:35 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0008</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0008
+Timestamp: 2026-04-27 00:25:28.867000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Revenant's Midnight Keeper
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with bat wing accents, containing a trapped swirling deep blue spirit flame, light refracting through cracked ghostly sapphire glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly sapphire glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Sapphire Glass, Deep Blue Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: revenant keeper, midnight lantern, sapphire glass, bat wing design, deep blue flame, grimdark collectible, spirit vessel, gothic decor, refractive lighting, internal glow, premium artifact
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0008_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:10:45 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0009</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0009
+Timestamp: 2026-04-27 00:25:31.624000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Lich's Phylactery Lantern
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with bone inlays, containing a trapped swirling amber spirit flame, light refracting through cracked ghostly topaz glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly topaz glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Topaz Glass, Amber Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: lich phylactery, amber flame, topaz glass, bone inlay, grimdark lantern, soul container, gothic artifact, undead relic, refractive depth, bioluminescent light, premium collectible
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0009_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:10:53 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0010</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0010
+Timestamp: 2026-04-27 00:25:34.871000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Wraith Warden's Cursed Beacon
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with raven motifs, containing a trapped swirling teal spirit flame, light refracting through cracked ghostly aquamarine glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly aquamarine glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Aquamarine Glass, Teal Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: wraith warden, cursed beacon, teal flame, aquamarine glass, raven motif, grimdark fantasy, spirit lantern, gothic collectible, refractive light, internal luminescence, premium design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0010_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:02 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0005</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0005
+Timestamp: 2026-04-27 00:22:44.870000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Arcane Archway of Forbidden Chronicles
+MJ_Prompt: An imposing archway fashioned from translucent moonstone and imperial jade positioned before a floating bibliotheca vault, preserved calfskin codices spiraling through the arcane gateway, ink-wash cosmic vapor intermixing with ancient paper essence, levitating brass charm shards etched with occult markings, cinematic chiaroscuro lighting with jade luminous aura, dark academia aesthetic, ultra-detailed moonstone translucency and brass esoteric mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: arcane archway, forbidden chronicles, translucent moonstone, jade aura, occult markings, floating vault, brass charms, dark academia collector, cosmic vapor, preserved codices, mentor-grade piece, esoteric design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0005_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:23:53 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0006</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0006
+Timestamp: 2026-04-27 00:22:49.443000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Ethereal Torii of Scholarly Ascension
+MJ_Prompt: A majestic torii structure composed of opalescent moonstone and imperial jade standing before an ascending knowledge repository, historical calfskin volumes flowing through the ethereal passage, ink-wash galaxy clouds fusing with manuscript vapor, floating brass amulet fragments inscribed with scholarly runes, cinematic chiaroscuro lighting with jade ethereal glow, dark academia aesthetic, ultra-detailed moonstone opalescence and brass scholarly mechanisms, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: ethereal torii, scholarly ascension, opalescent moonstone, jade glow, historical volumes, brass amulets, dark academia torii, galaxy atmosphere, knowledge repository, mentor design, scholarly runes, floating manuscripts
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0006_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:24:06 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0008</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0008
+Timestamp: 2026-04-27 00:22:57.794000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Mystic Threshold of Infinite Knowledge
+MJ_Prompt: A mystic threshold carved from luminescent moonstone and imperial jade placed before an infinite library expanse, timeless calfskin manuscripts orbiting through the mystical opening, ink-wash infinity clouds blending with aged book particles, floating brass rune fragments inscribed with infinite symbols, cinematic chiaroscuro lighting with jade mystical luminescence, dark academia aesthetic, ultra-detailed moonstone luminescence and brass infinite mechanisms, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: mystic threshold, infinite knowledge, luminescent moonstone, jade mysticism, timeless manuscripts, brass runes, dark academia mystique, infinity expanse, orbiting books, mentor artifact, infinite symbols, library realm
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0008_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:24:17 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0009</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0009
+Timestamp: 2026-04-27 00:23:01.621000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Sanctum Gate of Preserved Wisdom
+MJ_Prompt: A sanctified gate constructed from sacred moonstone and imperial jade standing before a preserved wisdom chamber, consecrated calfskin tomes circulating through the sanctum portal, ink-wash sacred clouds intermixing with preserved paper essence, levitating brass seal fragments etched with preservation glyphs, cinematic chiaroscuro lighting with jade sacred radiance, dark academia aesthetic, ultra-detailed moonstone sacred texture and brass preservation mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: sanctum gate, preserved wisdom, sacred moonstone, jade sanctification, consecrated tomes, brass seals, dark academia sanctum, preservation glyphs, wisdom chamber, mentor quality, sacred radiance, ancient preservation
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0009_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:24:32 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0010</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0010
+Timestamp: 2026-04-27 00:23:05.492000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Hermetic Portal of Ancient Codices
+MJ_Prompt: A hermetic portal structure formed from enigmatic moonstone and imperial jade positioned before a sealed codex vault, hermetic calfskin volumes spiraling through the sealed gateway, ink-wash hermetic clouds fusing with codex dust, floating brass cipher fragments inscribed with hermetic formulae, cinematic chiaroscuro lighting with jade hermetic glow, dark academia aesthetic, ultra-detailed moonstone enigmatic patterns and brass hermetic mechanisms, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: hermetic portal, ancient codices, enigmatic moonstone, jade hermetic, sealed vault, brass ciphers, dark academia hermetic, hermetic formulae, codex collection, mentor-grade portal, sealed knowledge, mystical gateway
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0010_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:24:45 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0011</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0011
+Timestamp: 2026-04-27 00:23:09.606000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Celestial Archway of Timeless Tomes
+MJ_Prompt: A celestial archway assembled from stellar moonstone and imperial jade rising before a timeless book repository, eternal calfskin manuscripts swirling through the celestial passage, ink-wash starfield clouds merging with timeless paper mist, hovering brass constellation fragments etched with stellar coordinates, cinematic chiaroscuro lighting with jade celestial luminosity, dark academia aesthetic, ultra-detailed moonstone stellar shimmer and brass celestial mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: celestial archway, timeless tomes, stellar moonstone, jade celestial, eternal manuscripts, brass constellations, dark academia celestial, starfield atmosphere, book repository, mentor collectible, stellar coordinates, cosmic library
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0011_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:25:04 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0013</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0013
+Timestamp: 2026-04-27 00:23:17.343000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Alchemist's Threshold of Transmuted Knowledge
+MJ_Prompt: An alchemist's threshold forged from alchemical moonstone and imperial jade standing before a transmutation library sanctum, alchemical calfskin formularies circulating through the transmutation gateway, ink-wash alchemical clouds intermixing with transmuted manuscript vapor, levitating brass formula fragments etched with transmutation symbols, cinematic chiaroscuro lighting with jade alchemical glow, dark academia aesthetic, ultra-detailed moonstone alchemical crystallization and brass transmutation mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: alchemist's threshold, transmuted knowledge, alchemical moonstone, jade alchemy, transmutation gateway, brass formulas, dark academia alchemy, alchemical symbols, formulary collection, mentor-grade alchemy, transmutation sanctum, mystical chemistry
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0013_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:25:22 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0014</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0014
+Timestamp: 2026-04-27 00:23:20.456000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Oracle's Portal of Prophetic Scriptures
+MJ_Prompt: An oracle's portal crafted from prophetic moonstone and imperial jade positioned before a divination archive realm, prophetic calfskin scrolls spiraling through the oracle gateway, ink-wash prophetic clouds fusing with divination parchment dust, floating brass prophecy fragments inscribed with oracular symbols, cinematic chiaroscuro lighting with jade prophetic luminescence, dark academia aesthetic, ultra-detailed moonstone prophetic iridescence and brass oracle mechanisms, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: oracle's portal, prophetic scriptures, prophetic moonstone, jade divination, oracle gateway, brass prophecy, dark academia oracle, oracular symbols, divination realm, mentor prophecy, prophetic scrolls, mystical foresight
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0014_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:25:33 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0011</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0011
+Timestamp: 2026-04-27 00:25:38.273000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Deathspeaker's Oracle Lamp
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with serpent coils, containing a trapped swirling orange spirit flame, light refracting through cracked ghostly carnelian glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly carnelian glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Carnelian Glass, Orange Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: deathspeaker lamp, oracle lantern, orange flame, carnelian glass, serpent coil, grimdark artifact, spirit light, gothic collectible, refractive glass, bioluminescent glow, premium fantasy
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0011_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:08 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0012</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0012
+Timestamp: 2026-04-27 00:25:41.140000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Phantom Lord's Caged Soul
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with crown spikes, containing a trapped swirling white spirit flame, light refracting through cracked ghostly opal glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly opal glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Opal Glass, White Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: phantom lord, caged soul, white flame, opal glass, crown spikes, grimdark lantern, spirit prison, gothic artifact, refractive depth, internal radiance, premium collectible
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0012_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:15 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0013</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0013
+Timestamp: 2026-04-27 00:25:45.576000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Gravekeepers Eternal Vigil
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with tombstone panels, containing a trapped swirling grey spirit flame, light refracting through cracked ghostly smoke glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly smoke glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Smoke Glass, Grey Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: gravekeeper vigil, grey flame, smoke glass, tombstone design, grimdark decor, eternal lantern, gothic artifact, spirit keeper, refractive light, bioluminescent core, premium fantasy
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0013_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:21 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0014</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0014
+Timestamp: 2026-04-27 00:25:47.853000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Soulbound Harbinger's Torch
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with wing embellishments, containing a trapped swirling magenta spirit flame, light refracting through cracked ghostly rose quartz glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly rose quartz glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Rose Quartz Glass, Magenta Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: harbinger torch, soulbound lantern, magenta flame, rose quartz glass, wing embellishment, grimdark collectible, spirit vessel, gothic decor, refractive lighting, internal glow, premium artifact
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0014_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:28 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0015</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0015
+Timestamp: 2026-04-27 00:25:50.709000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Cursed Monk's Penance Light
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with prayer scroll details, containing a trapped swirling yellow spirit flame, light refracting through cracked ghostly citrine glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly citrine glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Citrine Glass, Yellow Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: cursed monk, penance light, yellow flame, citrine glass, prayer scroll, grimdark lantern, spirit beacon, gothic artifact, refractive depth, bioluminescent glow, premium collectible
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0015_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:36 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0016</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0016
+Timestamp: 2026-04-27 00:25:53.211000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Shadowpriest's Ritual Vessel
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with ritual circle engravings, containing a trapped swirling indigo spirit flame, light refracting through cracked ghostly lapis glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly lapis glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Lapis Glass, Indigo Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: shadowpriest vessel, ritual lantern, indigo flame, lapis glass, ritual circle, grimdark fantasy, spirit container, gothic collectible, refractive light, internal radiance, premium design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0016_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:43 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0017</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0017
+Timestamp: 2026-04-27 00:26:06.574000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Dreadlord's Dominion Beacon
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with demonic horns, containing a trapped swirling scarlet spirit flame, light refracting through cracked ghostly garnet glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly garnet glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Garnet Glass, Scarlet Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: dreadlord beacon, dominion lantern, scarlet flame, garnet glass, demonic horns, grimdark artifact, spirit light, gothic collectible, refractive glass, bioluminescent core, premium fantasy
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0017_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:50 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0018</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0018
+Timestamp: 2026-04-27 00:26:09.802000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Sepulcher Guardian's Flame
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with crypt door motifs, containing a trapped swirling turquoise spirit flame, light refracting through cracked ghostly turquoise glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly turquoise glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Turquoise Glass, Turquoise Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: sepulcher guardian, crypt lantern, turquoise flame, turquoise glass, crypt door motif, grimdark decor, spirit vessel, gothic artifact, refractive depth, internal luminescence, premium collectible
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0018_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:11:58 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0019</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0019
+Timestamp: 2026-04-27 00:26:11.578000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Abyssal Watcher's Eternal Eye
+MJ_Prompt: An ornate gothic lantern made of heavy wrought iron with eye socket frame, containing a trapped swirling cyan spirit flame, light refracting through cracked ghostly aqua glass, grimdark aesthetic, high contrast shadows, macro photography, isolated on white background, wrought iron and ghostly aqua glass materials, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Ghostly Aqua Glass, Cyan Spirit Flame, Gothic Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: abyssal watcher, eternal eye, cyan flame, aqua glass, eye socket design, grimdark lantern, spirit beacon, gothic collectible, refractive lighting, bioluminescent glow, premium artifact
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0019_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:12:04 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0021</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0021
+Timestamp: 2026-04-27 00:26:54.911000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Emerald Despair Lantern
+MJ_Prompt: A corrupted gothic lantern forged from blackened wrought iron with razor-sharp filigree, containing a violent emerald spirit flame thrashing against frosted jade-tinted glass, grimdark aesthetic, dramatic side lighting, isolated on white background, oxidized iron and emerald glass materials, hyper-detailed mentor-grade object design, primary material system: Blackened Wrought Iron, Jade-Tinted Glass, Emerald Spirit Flame, Sharp Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: grimdark lantern, emerald spirit flame, gothic ironwork, frosted jade glass, corrupted artifact, dark fantasy decor, mentor-grade collectible, bioluminescent glow, premium gothic lantern, wrought iron filigree
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0021_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:12:13 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0022</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0022
+Timestamp: 2026-04-27 00:26:58.581000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Violet Torment Lantern
+MJ_Prompt: A corrupted gothic lantern forged from blackened wrought iron with razor-sharp filigree, containing a violent violet spirit flame thrashing against frosted amethyst-tinted glass, grimdark aesthetic, dramatic side lighting, isolated on white background, oxidized iron and violet glass materials, hyper-detailed mentor-grade object design, primary material system: Blackened Wrought Iron, Amethyst-Tinted Glass, Violet Spirit Flame, Sharp Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: violet flame lantern, amethyst gothic decor, corrupted spirit vessel, blackened iron filigree, dark fantasy artifact, grimdark collectible, translucent depth lighting, premium lantern design, wrought iron craftsmanship, bioluminescent accent
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0022_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:12:22 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0023</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0023
+Timestamp: 2026-04-27 00:27:01.310000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Azure Suffering Lantern
+MJ_Prompt: A corrupted gothic lantern forged from blackened wrought iron with razor-sharp filigree, containing a violent azure spirit flame thrashing against frosted sapphire-tinted glass, grimdark aesthetic, dramatic side lighting, isolated on white background, oxidized iron and blue glass materials, hyper-detailed mentor-grade object design, primary material system: Blackened Wrought Iron, Sapphire-Tinted Glass, Azure Spirit Flame, Sharp Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: azure spirit lantern, sapphire gothic glass, corrupted flame vessel, dark fantasy ironwork, grimdark blue lantern, premium collectible artifact, blackened wrought iron, translucent depth, museum-grade lighting, bioluminescent core
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0023_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:12:31 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0024</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0024
+Timestamp: 2026-04-27 00:27:05.073000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Obsidian Wrath Lantern
+MJ_Prompt: A corrupted gothic lantern forged from blackened wrought iron with razor-sharp filigree, containing a violent obsidian spirit flame thrashing against frosted smoke-tinted glass, grimdark aesthetic, dramatic side lighting, isolated on white background, oxidized iron and dark glass materials, hyper-detailed mentor-grade object design, primary material system: Blackened Wrought Iron, Smoke-Tinted Glass, Obsidian Spirit Flame, Sharp Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: obsidian flame lantern, smoke glass gothic, dark spirit vessel, corrupted ironwork, grimdark black lantern, mentor-grade artifact, wrought iron filigree, translucent smoke effect, premium dark fantasy, bioluminescent shadow
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0024_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:12:41 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0025</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0025
+Timestamp: 2026-04-27 00:27:07.908000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Amber Anguish Lantern
+MJ_Prompt: A corrupted gothic lantern forged from blackened wrought iron with razor-sharp filigree, containing a violent amber spirit flame thrashing against frosted honey-tinted glass, grimdark aesthetic, dramatic side lighting, isolated on white background, oxidized iron and amber glass materials, hyper-detailed mentor-grade object design, primary material system: Blackened Wrought Iron, Honey-Tinted Glass, Amber Spirit Flame, Sharp Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: amber spirit lantern, honey glass gothic, corrupted flame artifact, blackened iron decor, grimdark warm lantern, premium collectible design, wrought iron craftsmanship, translucent amber depth, dark fantasy lighting, bioluminescent warmth
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0025_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:12:48 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0026</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0026
+Timestamp: 2026-04-27 00:27:11.159000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Frost Agony Lantern
+MJ_Prompt: A corrupted gothic lantern forged from blackened wrought iron with razor-sharp filigree, containing a violent ice-white spirit flame thrashing against frosted crystal-tinted glass, grimdark aesthetic, dramatic side lighting, isolated on white background, oxidized iron and frost glass materials, hyper-detailed mentor-grade object design, primary material system: Blackened Wrought Iron, Crystal-Tinted Glass, Ice-White Spirit Flame, Sharp Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: frost flame lantern, ice white spirit, crystal gothic glass, corrupted winter artifact, grimdark frozen lantern, premium ironwork collectible, translucent frost depth, dark fantasy ice, wrought iron filigree, bioluminescent cold
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0026_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:12:56 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0027</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0027
+Timestamp: 2026-04-27 00:27:14.469000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Magenta Malice Lantern
+MJ_Prompt: A corrupted gothic lantern forged from blackened wrought iron with razor-sharp filigree, containing a violent magenta spirit flame thrashing against frosted rose-tinted glass, grimdark aesthetic, dramatic side lighting, isolated on white background, oxidized iron and magenta glass materials, hyper-detailed mentor-grade object design, primary material system: Blackened Wrought Iron, Rose-Tinted Glass, Magenta Spirit Flame, Sharp Filigree, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: magenta spirit lantern, rose gothic glass, corrupted pink flame, blackened iron artifact, grimdark vibrant lantern, mentor-grade collectible, wrought iron design, translucent magenta depth, premium fantasy decor, bioluminescent rose
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0027_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:13:04 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0028</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0028
+Timestamp: 2026-04-27 00:28:59.944000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Obsidian Shrine Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with obsidian shrine gate frame, moonstone inlays, containing swirling violet-white spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft celestial glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Obsidian, Moonstone, Imperial Jade Glass, Talisman Fragments, Violet-White Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: grimdark lantern, soul vessel, obsidian shrine, spirit flame, talisman fragments, jade glass, moonstone inlay, gothic artifact, ethereal glow, mentor-grade collectible, acrylic display piece
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0028_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:13:13 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0030</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0030
+Timestamp: 2026-04-27 00:29:06.519000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Spectral Temple Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron temple gate frame, opal inlays, containing swirling cyan-silver spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft spectral glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Opal, Imperial Jade Glass, Talisman Fragments, Cyan-Silver Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: spectral lantern, temple gate, opal inlay, cyan flame, soul vessel, jade glass, grimdark collectible, wrought iron frame, talisman fragments, ethereal light, mentor-grade artifact
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0030_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:13:23 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0031</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0031
+Timestamp: 2026-04-27 00:29:09.805000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Midnight Sanctuary Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron sanctuary arch frame, black pearl inlays, containing swirling indigo-white spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft midnight glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Black Pearl, Imperial Jade Glass, Talisman Fragments, Indigo-White Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: midnight soul lantern, sanctuary arch, black pearl, indigo flame, grimdark design, jade glass, wrought iron, talisman magic, gothic artifact, premium display, acrylic collectible
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0031_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:13:33 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0032</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0032
+Timestamp: 2026-04-27 00:29:12.708000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Amber Monastery Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron monastery gate frame, amber crystal inlays, containing swirling golden-orange spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft amber glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Amber Crystal, Imperial Jade Glass, Talisman Fragments, Golden-Orange Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: amber soul lantern, monastery gate, golden flame, amber crystal, jade glass panels, grimdark collectible, wrought iron, talisman fragments, gothic aesthetic, mentor-grade design, acrylic art
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0032_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:13:40 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0033</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0033
+Timestamp: 2026-04-27 00:29:18.252000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Ethereal Archway Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron archway silhouette frame, selenite inlays, containing swirling pearl-white spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft ethereal glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Selenite, Imperial Jade Glass, Talisman Fragments, Pearl-White Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: ethereal lantern, archway frame, selenite crystal, pearl flame, soul vessel, jade glass, grimdark artifact, wrought iron, talisman magic, gothic collectible, premium acrylic display
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0033_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:13:49 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0034</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0034
+Timestamp: 2026-04-27 00:29:22.525000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Emerald Sanctum Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron sanctum gate frame, emerald inlays, containing swirling green-white spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft verdant glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Emerald, Imperial Jade Glass, Talisman Fragments, Green-White Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: emerald soul lantern, sanctum gate, green flame, emerald inlay, jade glass, grimdark design, wrought iron frame, talisman fragments, gothic artifact, mentor-grade collectible, acrylic piece
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0034_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:13:57 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0035</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0035
+Timestamp: 2026-04-27 00:29:24.404000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Twilight Portal Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron portal frame, labradorite inlays, containing swirling purple-blue spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft twilight glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Labradorite, Imperial Jade Glass, Talisman Fragments, Purple-Blue Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: twilight lantern, portal frame, labradorite inlay, purple flame, soul vessel, jade glass panels, grimdark collectible, wrought iron, talisman magic, gothic design, premium acrylic art
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0035_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:14:07 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0036</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0036
+Timestamp: 2026-04-27 00:29:25.568000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Frost Cathedral Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron cathedral gate frame, aquamarine inlays, containing swirling ice-blue spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft frost glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Aquamarine, Imperial Jade Glass, Talisman Fragments, Ice-Blue Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: frost soul lantern, cathedral gate, aquamarine crystal, ice-blue flame, jade glass, grimdark aesthetic, wrought iron, talisman fragments, gothic artifact, mentor-grade display, acrylic collectible
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0036_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:14:17 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0037</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0037
+Timestamp: 2026-04-27 00:29:27.322000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Onyx Shrine Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron shrine torii frame, onyx inlays, containing swirling black-silver spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft shadow glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Onyx, Imperial Jade Glass, Talisman Fragments, Black-Silver Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: onyx soul lantern, shrine torii, black flame, onyx inlay, jade glass panels, grimdark collectible, wrought iron frame, talisman magic, gothic design, premium artifact, acrylic display
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0037_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:14:25 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0038</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0038
+Timestamp: 2026-04-27 00:29:30.124000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Rose Quartz Chapel Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron chapel gate frame, rose quartz inlays, containing swirling pink-white spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft rose glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Rose Quartz, Imperial Jade Glass, Talisman Fragments, Pink-White Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: rose quartz lantern, chapel gate, pink flame, rose quartz inlay, soul vessel, jade glass, grimdark artifact, wrought iron, talisman fragments, gothic collectible, mentor-grade acrylic
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0038_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:14:32 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0039</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0039
+Timestamp: 2026-04-27 00:29:32.948000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Sapphire Temple Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron temple archway frame, sapphire inlays, containing swirling deep-blue spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft sapphire glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Sapphire, Imperial Jade Glass, Talisman Fragments, Deep-Blue Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: sapphire soul lantern, temple archway, deep-blue flame, sapphire inlay, jade glass panels, grimdark design, wrought iron, talisman magic, gothic artifact, premium collectible, acrylic display
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0039_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:14:40 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Acrylic-Grimdark-0040</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Acrylic-Grimdark-0040
+Timestamp: 2026-04-27 00:29:35.368000
+Category: Grimdark
+Product_Type: Acrylic
+Style: Grimdark Mentor-Grade
+Title: Silver Moon Gate Soul Lantern
+MJ_Prompt: An ethereal gothic lantern with wrought iron moon gate silhouette frame, moonstone inlays, containing swirling silver-white spirit flame with floating talisman fragments, ink-wash nebula patterns on imperial jade glass panels, grimdark aesthetic, soft lunar glow, isolated on white background, hyper-detailed mentor-grade object design, primary material system: Wrought Iron, Moonstone, Imperial Jade Glass, Talisman Fragments, Silver-White Flame, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, 3D depth, refractive light, internal glow, ray tracing, --ar 2:3 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: silver moon lantern, moon gate, lunar flame, moonstone inlay, soul vessel, jade glass, grimdark collectible, wrought iron frame, talisman fragments, gothic aesthetic, mentor-grade acrylic
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Acrylic\Photo-Block\MASTER_Acrylic-Grimdark-0040_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>5/4/2026  8:14:48 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0017</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0017
+Timestamp: 2026-04-27 00:23:32.693000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Magister's Torii of Academic Mastery
+MJ_Prompt: A magister's torii fashioned from academic moonstone and imperial jade positioned before a mastery library pinnacle, masterwork calfskin treatises orbiting through the magister's gateway, ink-wash academic clouds intermixing with mastery parchment vapor, floating brass mastery fragments etched with magisterial symbols, cinematic chiaroscuro lighting with jade academic radiance, dark academia aesthetic, ultra-detailed moonstone academic crystallization and brass magisterial mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: magister's torii, academic mastery, academic moonstone, jade magisterial, mastery library, brass symbols, dark academia master, magisterial gateway, masterwork treatises, mentor mastery, academic pinnacle, scholarly excellence
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0017_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:25:58 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0019</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0019
+Timestamp: 2026-04-27 00:23:43.018000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Archivist's Gateway of Catalogued Eternity
+MJ_Prompt: An archivist's gateway carved from cataloguing moonstone and imperial jade standing before an eternal classification chamber, catalogued calfskin indices flowing through the archivist's passage, ink-wash classification clouds merging with catalogued page essence, levitating brass index fragments etched with archival notations, cinematic chiaroscuro lighting with jade archival luminescence, dark academia aesthetic, ultra-detailed moonstone cataloguing patterns and brass archival mechanisms, hyper-detailed mentor-grade artifact design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: archivist's gateway, catalogued eternity, cataloguing moonstone, jade archival, classification chamber, brass indices, dark academia archivist, archival notations, eternal catalogue, mentor archivist, organized knowledge, systematic wisdom
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0019_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:26:14 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0020</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0020
+Timestamp: 2026-04-27 00:23:48.990000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Mentor's Threshold of Transcendent Learning
+MJ_Prompt: A mentor's threshold wrought from transcendent moonstone and imperial jade positioned before an enlightenment library expanse, transcendent calfskin teachings circulating through the mentor's portal, ink-wash transcendent clouds blending with enlightenment manuscript vapor, floating brass enlightenment fragments inscribed with mentorial wisdom, cinematic chiaroscuro lighting with jade transcendent radiance, dark academia aesthetic, ultra-detailed moonstone transcendent shimmer and brass mentorial mechanisms, hyper-detailed mentor-grade object design, primary material system: Moonstone, Imperial Jade, Ancient Calfskin, Burnished Brass, Ink-wash Nebula, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: mentor's threshold, transcendent learning, transcendent moonstone, jade enlightenment, mentor portal, brass wisdom, dark academia mentor, mentorial teachings, enlightenment expanse, mentor-grade excellence, transcendent knowledge, ultimate wisdom
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0020_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:26:26 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0021</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0021
+Timestamp: 2026-04-27 00:23:58.101000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Celestial Chronometer Archive Sphere
+MJ_Prompt: A massive spherical archive vessel constructed from corroded brass and fractured observatory glass containing gravity-defying ancient astronomical books, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating leather-bound star charts, swirling celestial parchment dust trapped inside the sphere, brass clockwork meridian rings, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Brass, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Leather, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: dark academia poster, alchemical vessel art, celestial library aesthetic, corroded brass sphere, kintsugi gold repair, bioluminescent books, astronomical archive, vintage chronometer design, mentor-grade collectible, immersive dark academia
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0021_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:26:42 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0022</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0022
+Timestamp: 2026-04-27 00:24:01.823000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Temporal Reliquary Bell Jar
+MJ_Prompt: A towering bell jar reliquary constructed from corroded iron and cracked crystal containing gravity-defying ancient chronology manuscripts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating vellum pages, swirling temporal parchment dust trapped inside the vessel, brass clockwork pressure gauges, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, Cracked Crystal, Kintsugi Gold, Toxic Jade, Ancient Vellum, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: temporal library art, bell jar reliquary, dark academia decor, corroded iron vessel, kintsugi crystal repair, chronology manuscripts, jade bioluminescence, mentor-grade poster, vintage scientific aesthetic, immersive composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0022_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:26:54 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0023</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0023
+Timestamp: 2026-04-27 00:24:05.175000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Hermetic Knowledge Lantern
+MJ_Prompt: A monumental hermetic lantern constructed from corroded copper and cracked glass panels containing gravity-defying ancient hermetic texts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating aged parchment pages, swirling alchemical dust trapped inside the lantern, brass clockwork ventilation system, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Copper, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Parchment, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: hermetic lantern art, dark academia poster, corroded copper vessel, ancient text container, kintsugi gold seams, jade bioluminescence, alchemical aesthetic, mentor-grade design, immersive library decor, cinematic lighting
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0023_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:27:08 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0024</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0024
+Timestamp: 2026-04-27 00:24:08.854000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Bibliotheca Pressure Chamber
+MJ_Prompt: A massive industrial pressure chamber constructed from corroded iron and cracked reinforced glass containing gravity-defying ancient library volumes, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating leather-bound tomes, swirling bibliographic dust trapped inside the chamber, brass clockwork pressure release valves, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Leather, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: industrial library chamber, pressure vessel art, dark academia aesthetic, corroded iron design, kintsugi repair gold, bioluminescent books, bibliotheca poster, mentor-grade collectible, immersive composition, vintage scientific
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0024_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:27:21 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0025</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0025
+Timestamp: 2026-04-27 00:24:13.339000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Chrono-Codex Terrarium
+MJ_Prompt: A grand terrarium vessel constructed from corroded bronze and cracked glass containing gravity-defying ancient time-keeping manuscripts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating calfskin folios, swirling chronological parchment dust trapped inside the terrarium, brass clockwork humidity regulators, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Bronze, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Calfskin, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: chronological terrarium art, time-keeping codex, dark academia poster, corroded bronze vessel, kintsugi gold veins, jade bioluminescence, manuscript container, mentor-grade design, immersive library aesthetic, cinematic composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0025_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:27:33 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0026</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0026
+Timestamp: 2026-04-27 00:24:15.539000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Apothecary Archive Cylinder
+MJ_Prompt: A towering cylindrical archive constructed from corroded iron and cracked apothecary glass containing gravity-defying ancient pharmaceutical texts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating medicinal parchment pages, swirling herbal dust trapped inside the cylinder, brass clockwork dosage mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Parchment, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: apothecary cylinder art, pharmaceutical archive, dark academia decor, corroded iron vessel, kintsugi repair seams, jade bioluminescence, medicinal texts, mentor-grade poster, vintage medical aesthetic, immersive design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0026_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:27:55 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0027</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0027
+Timestamp: 2026-04-27 00:24:18.455000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Astrolabe Knowledge Dome
+MJ_Prompt: A magnificent dome vessel constructed from corroded brass and cracked observatory glass containing gravity-defying ancient astrolabe manuscripts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating astronomical vellum, swirling celestial calculation dust trapped inside the dome, brass clockwork armillary mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Brass, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Vellum, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: astrolabe dome art, astronomical archive, dark academia poster, corroded brass vessel, kintsugi gold repair, celestial manuscripts, jade bioluminescence, mentor-grade collectible, observatory aesthetic, immersive composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0027_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:28:12 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0028</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0028
+Timestamp: 2026-04-27 00:24:23.501000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Alchemist's Retort Library
+MJ_Prompt: A massive alchemical retort constructed from corroded copper and cracked laboratory glass containing gravity-defying ancient alchemy books, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating transmutation pages, swirling metallic parchment dust trapped inside the retort, brass clockwork distillation valves, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Copper, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Calfskin, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: alchemical retort art, transmutation library, dark academia aesthetic, corroded copper vessel, kintsugi repair gold, jade bioluminescence, alchemy manuscripts, mentor-grade poster, laboratory vintage design, immersive environment
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0028_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:28:39 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0030</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0030
+Timestamp: 2026-04-27 00:24:29.777000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Grimoire Preservation Capsule
+MJ_Prompt: A towering preservation capsule constructed from corroded bronze and cracked preservation glass containing gravity-defying ancient grimoire volumes, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating spell parchment pages, swirling mystical dust trapped inside the capsule, brass clockwork sealing mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Bronze, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Calfskin, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: grimoire capsule art, spell book preservation, dark academia decor, corroded bronze vessel, kintsugi repair seams, mystical manuscripts, jade bioluminescence, mentor-grade poster, occult aesthetic, immersive design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0030_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:29:01 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0031</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0031
+Timestamp: 2026-04-27 00:24:30.986000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Botanical Codex Conservatory
+MJ_Prompt: A grand conservatory vessel constructed from corroded iron and cracked botanical glass containing gravity-defying ancient herbarium books, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating pressed plant pages, swirling botanical parchment dust trapped inside the conservatory, brass clockwork climate control valves, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Vellum, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: botanical conservatory art, herbarium codex, dark academia poster, corroded iron vessel, kintsugi gold repair, plant manuscripts, jade bioluminescence, mentor-grade collectible, naturalist aesthetic, immersive composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0031_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:29:22 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0032</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0032
+Timestamp: 2026-04-27 00:24:33.826000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Observatory Archive Prism
+MJ_Prompt: A massive prismatic archive constructed from corroded brass and cracked optical glass containing gravity-defying ancient astronomy texts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating star chart parchment, swirling cosmic dust trapped inside the prism, brass clockwork lens adjustment mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Brass, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Parchment, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: observatory prism art, astronomical archive, dark academia aesthetic, corroded brass vessel, kintsugi repair gold, star chart manuscripts, jade bioluminescence, mentor-grade poster, optical design, immersive environment
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0032_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:29:50 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0033</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0033
+Timestamp: 2026-04-27 00:24:36.642000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Philosophical Theorem Reliquary
+MJ_Prompt: A monumental reliquary constructed from corroded iron and cracked philosophical glass containing gravity-defying ancient philosophy manuscripts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating theorem parchment pages, swirling intellectual dust trapped inside the reliquary, brass clockwork logic mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Calfskin, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: philosophical reliquary art, theorem manuscripts, dark academia poster, corroded iron vessel, kintsugi gold seams, ancient philosophy texts, jade bioluminescence, mentor-grade design, intellectual aesthetic, immersive composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0033_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:30:07 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0034</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0034
+Timestamp: 2026-04-27 00:24:39.915000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Nautical Archive Barometer
+MJ_Prompt: A towering barometer vessel constructed from corroded copper and cracked maritime glass containing gravity-defying ancient navigation books, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating sea chart pages, swirling oceanic parchment dust trapped inside the barometer, brass clockwork pressure measurement systems, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Copper, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Leather, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: nautical barometer art, maritime archive, dark academia decor, corroded copper vessel, kintsugi repair gold, navigation manuscripts, jade bioluminescence, mentor-grade poster, seafaring aesthetic, immersive design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0034_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>5/4/2026  10:30:24 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Etsy digital gray launch safeguards
</commit_message>
<xml_diff>
--- a/Database/Etsy_listing.xlsx
+++ b/Database/Etsy_listing.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E241"/>
+  <dimension ref="A1:E249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9083,6 +9083,294 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0035</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0035
+Timestamp: 2026-04-27 00:24:42.773000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Theological Codex Sanctuary
+MJ_Prompt: A magnificent sanctuary vessel constructed from corroded bronze and cracked cathedral glass containing gravity-defying ancient theological texts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating sacred vellum pages, swirling devotional parchment dust trapped inside the sanctuary, brass clockwork prayer mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Bronze, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Vellum, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: theological sanctuary art, sacred codex vessel, dark academia poster, corroded bronze design, kintsugi gold veins, ancient religious texts, jade bioluminescence, mentor-grade collectible, cathedral aesthetic, immersive composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0035_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>5/6/2026  5:49:57 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0036</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0036
+Timestamp: 2026-04-27 00:24:45.692000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Mechanical Encyclopedia Sphere
+MJ_Prompt: A massive spherical encyclopedia constructed from corroded iron and cracked technical glass containing gravity-defying ancient engineering books, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating blueprint parchment, swirling mechanical dust trapped inside the sphere, brass clockwork gear display systems, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Calfskin, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: mechanical encyclopedia sphere, engineering archive, dark academia aesthetic, corroded iron vessel, kintsugi repair seams, blueprint manuscripts, jade bioluminescence, mentor-grade poster, industrial design, immersive environment
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0036_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>5/6/2026  5:50:05 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0037</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0037
+Timestamp: 2026-04-27 00:24:48.901000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Cryptographic Vault Cylinder
+MJ_Prompt: A towering cylindrical vault constructed from corroded brass and cracked cipher glass containing gravity-defying ancient cryptography manuscripts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating encoded parchment pages, swirling symbolic dust trapped inside the cylinder, brass clockwork encryption mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Brass, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Parchment, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: cryptographic vault art, cipher manuscript archive, dark academia poster, corroded brass cylinder, kintsugi gold repair, encoded texts, jade bioluminescence, mentor-grade design, secret knowledge aesthetic, immersive composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0037_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>5/6/2026  5:50:11 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0038</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0038
+Timestamp: 2026-04-27 00:24:52.242000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Geological Archive Geode
+MJ_Prompt: A monumental geode vessel constructed from corroded iron and cracked mineral glass containing gravity-defying ancient geology texts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating stone catalog pages, swirling crystalline parchment dust trapped inside the geode, brass clockwork specimen rotation systems, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Iron, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Vellum, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: geological geode archive, mineral manuscript art, dark academia decor, corroded iron vessel, kintsugi repair gold, stone catalog texts, jade bioluminescence, mentor-grade poster, naturalist aesthetic, immersive design
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0038_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>5/6/2026  7:19:04 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0039</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0039
+Timestamp: 2026-04-27 00:24:54.966000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Horological Manuscript Chamber
+MJ_Prompt: A grand chamber vessel constructed from corroded bronze and cracked timepiece glass containing gravity-defying ancient horology books, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating clockwork parchment pages, swirling temporal dust trapped inside the chamber, brass clockwork escapement mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Bronze, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Calfskin, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: horological chamber art, timepiece manuscript archive, dark academia poster, corroded bronze vessel, kintsugi gold seams, clockwork texts, jade bioluminescence, mentor-grade collectible, watchmaker aesthetic, immersive composition
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0039_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>5/6/2026  7:19:10 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0040</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0040
+Timestamp: 2026-04-27 00:24:58.086000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Meteorological Archive Orrery
+MJ_Prompt: A massive orrery archive constructed from corroded copper and cracked atmospheric glass containing gravity-defying ancient weather manuscripts, kintsugi repair seams glowing with golden light, toxic jade bioluminescence illuminating meteorological parchment, swirling climatic dust trapped inside the orrery, brass clockwork atmospheric prediction mechanisms, dramatic side lighting with emerald glow, dark academia aesthetic, ultra-detailed corrosion and glass fracture patterns, hyper-detailed mentor-grade object design, primary material system: Corroded Copper, Cracked Glass, Kintsugi Gold, Toxic Jade, Ancient Parchment, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: meteorological orrery art, weather manuscript archive, dark academia aesthetic, corroded copper vessel, kintsugi repair gold, atmospheric texts, jade bioluminescence, mentor-grade poster, scientific design, immersive environment
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0040_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>5/6/2026  7:19:16 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0041</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0041
+Timestamp: 2026-04-27 00:32:18.321000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Obsidian Eclipse Astrological Globe
+MJ_Prompt: A triple-ringed astrological globe with obsidian meridian rings, starlight jade sphere core displaying constellations in silver filigree, crystalline star charts orbiting in concentric layers, floating stardust nodes suspended in zero gravity, dark oak pedestal base with astronomical engravings in gold leaf, academia study aesthetic, warm candlelight from left casting dramatic shadows, hyper-detailed mentor-grade object design, primary material system: Obsidian, Starlight Jade, Dark Oak, Gold Leaf, Crystalline Glass, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: celestial globe, astrological artifact, obsidian decor, academia aesthetic, constellation map, starlight jade, luxury collectible, astronomical instrument, mentor-grade design, museum-quality artifact, handcrafted globe
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0041_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>5/6/2026  7:19:24 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Poster-Academia-0042</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID: Poster-Academia-0042
+Timestamp: 2026-04-27 00:32:22.522000
+Category: Academia
+Product_Type: Poster
+Style: Academia Mentor-Grade
+Title: Midnight Constellation Armillary Sphere
+MJ_Prompt: A quadruple-ringed armillary sphere with obsidian orbital bands, starlight jade celestial core etched with zodiac symbols in platinum inlay, crystalline ecliptic rings rotating in perfect alignment, suspended meteor fragments in gravitational balance, dark oak foundation with carved lunar phases in gold leaf, scholarly library atmosphere, warm candlelight from left creating long shadows, hyper-detailed mentor-grade object design, primary material system: Obsidian, Starlight Jade, Dark Oak, Gold Leaf, Crystalline Glass, micro-engraved surface relief, visible handcrafted edge bevels, layered translucent depth, subtle internal bioluminescent glow, refined kintsugi-like vein logic, floating accent fragments arranged with intentional negative space, cinematic rim lighting plus soft museum-grade overhead fill, crisp silhouette readability, centered premium product composition, clean contour separation, high-end collectible artifact aesthetic, isolated on white background, full frame, cinematic lighting, edge-to-edge composition, immersive environment, --ar 9:16 --v 6.1 --style raw --no skin, person, text, watermark
+SEO_Hook: armillary sphere, zodiac symbols, obsidian rings, celestial navigation, starlight jade core, platinum inlay, scholarly decor, astronomical model, luxury artifact, handcrafted instrument, museum piece
+Status: Completed
+</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>C:\AIprojects\openclaw_difi\Output\Poster\Premium-Matte-Vertical\MASTER_Poster-Academia-0042_Ready_for_Steaming\Production_Design.png</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>5/6/2026  7:19:30 PM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>